<commit_message>
moved the consolidated methods to coreframework, removed all the usage of Attachment method, Completed three Payment request Test Cases
</commit_message>
<xml_diff>
--- a/src/main/resources/PaymentRequest_Field_Values.xlsx
+++ b/src/main/resources/PaymentRequest_Field_Values.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{3C6B5F0E-19AD-46E6-BF2E-01B31D2048A5}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{4A753B77-D850-4D4A-BA08-4D6E3FD0B859}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="1" xr2:uid="{3DB20064-4C88-40D6-9C39-740182FAD6DF}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="2" xr2:uid="{3DB20064-4C88-40D6-9C39-740182FAD6DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Adhoc Reimbursement Creation" sheetId="1" r:id="rId1"/>
     <sheet name="Edition" sheetId="2" r:id="rId2"/>
+    <sheet name="Paid Details" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="17">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -62,6 +63,21 @@
   </si>
   <si>
     <t>Checked</t>
+  </si>
+  <si>
+    <t>CheckNumber__c</t>
+  </si>
+  <si>
+    <t>VoucherNumber__c</t>
+  </si>
+  <si>
+    <t>PaidDate__c</t>
+  </si>
+  <si>
+    <t>PaymentReference__c</t>
+  </si>
+  <si>
+    <t>Nil</t>
   </si>
 </sst>
 </file>
@@ -510,4 +526,74 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B525EBA-C08E-4BA7-8EAD-8589568CEF96}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2">
+        <v>6789678654</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3">
+        <v>5678</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged PR 2114: Merge MahadevProduct18March to master
Fixed issues in funding source and scheduled payment request
</commit_message>
<xml_diff>
--- a/src/main/resources/PaymentRequest_Field_Values.xlsx
+++ b/src/main/resources/PaymentRequest_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCFBAED8-7C78-4A28-9863-37BCC626668E}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DCE0D61-E27D-418B-A4E6-21DC32BF7DE9}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{3DB20064-4C88-40D6-9C39-740182FAD6DF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{3DB20064-4C88-40D6-9C39-740182FAD6DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Adhoc Reimbursement Creation" sheetId="1" r:id="rId1"/>
@@ -440,13 +440,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{493C7654-D1A3-4E56-B510-F05D117ABEF1}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,7 +457,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -476,14 +476,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20A3052A-53B6-4404-9922-9D5C64B8A322}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.21875" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -494,7 +494,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -505,7 +505,7 @@
         <v>78954</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -516,7 +516,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -527,7 +527,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -546,13 +546,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC07F6C2-F9EE-4A78-8EFB-9F3B27056F73}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -563,7 +563,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -574,7 +574,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -585,7 +585,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -605,13 +605,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B525EBA-C08E-4BA7-8EAD-8589568CEF96}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -622,7 +622,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -633,7 +633,7 @@
         <v>6789678654</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -644,7 +644,7 @@
         <v>5678</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -655,7 +655,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
refactored payment request and closeout module grantor
</commit_message>
<xml_diff>
--- a/src/main/resources/PaymentRequest_Field_Values.xlsx
+++ b/src/main/resources/PaymentRequest_Field_Values.xlsx
@@ -1,26 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21425"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DCE0D61-E27D-418B-A4E6-21DC32BF7DE9}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4505"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{3DB20064-4C88-40D6-9C39-740182FAD6DF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Adhoc Reimbursement Creation" sheetId="1" r:id="rId1"/>
     <sheet name="Advance Edition" sheetId="4" r:id="rId2"/>
     <sheet name="Edition" sheetId="2" r:id="rId3"/>
     <sheet name="Paid Details" sheetId="3" r:id="rId4"/>
+    <sheet name="No Program Income_Edition" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="179017"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="124519"/>
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -28,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="18">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -87,8 +82,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,7 +180,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -237,7 +232,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -431,22 +426,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{493C7654-D1A3-4E56-B510-F05D117ABEF1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,7 +452,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -474,16 +469,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20A3052A-53B6-4404-9922-9D5C64B8A322}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.28515625" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -494,7 +489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -505,7 +500,7 @@
         <v>78954</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -516,7 +511,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -527,7 +522,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -544,15 +539,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC07F6C2-F9EE-4A78-8EFB-9F3B27056F73}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -563,7 +558,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -574,7 +569,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -585,7 +580,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -603,15 +598,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B525EBA-C08E-4BA7-8EAD-8589568CEF96}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -622,7 +617,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -633,7 +628,7 @@
         <v>6789678654</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -644,7 +639,7 @@
         <v>5678</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -655,7 +650,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -670,4 +665,51 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>